<commit_message>
Onboard SpiceJet under the Ancillaries supplier feature; Admin and Portal runs
- Supplier spicejet (supplier.json, SupplierChecklist rev 11), registry updates
- Runner: SpiceJet seat/booking handling, unique test data (docs.js), leg-space
  rule groups 20-22, Admin PNR Query in its own login window, Admin pay-after-hold
  path, report paging over every page, PNR Query parse fixes (+ tests),
  longer seat-map wait
- Suite: TC-SM-LEG-001..005
- Runs 015 (Admin) and 016 (Portal) with logs, screenshots and reports

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/platform_core_data/supplier-features/ancillaries/shared/ancillaries-baseline/test_design/TestCases_AncillariesSeatMap.xlsx
+++ b/platform_core_data/supplier-features/ancillaries/shared/ancillaries-baseline/test_design/TestCases_AncillariesSeatMap.xlsx
@@ -678,7 +678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T125"/>
+  <dimension ref="A1:T130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -10747,13 +10747,423 @@
         </is>
       </c>
     </row>
-    <row r="126" ht="150" customHeight="1"/>
-    <row r="127" ht="150" customHeight="1"/>
-    <row r="128" ht="150" customHeight="1"/>
-    <row r="129" ht="150" customHeight="1"/>
-    <row r="130" ht="150" customHeight="1"/>
+    <row r="126" ht="150" customHeight="1">
+      <c r="A126" s="2" t="n">
+        <v>125</v>
+      </c>
+      <c r="B126" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-SM-LEG-001</t>
+        </is>
+      </c>
+      <c r="C126" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y. Leg space seats</t>
+        </is>
+      </c>
+      <c r="D126" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A child CAN select a leg space seat on the seat map</t>
+        </is>
+      </c>
+      <c r="E126" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A child may have a leg space seat; only an adult holding an infant is restricted.</t>
+        </is>
+      </c>
+      <c r="F126" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="G126" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">See the 'Before every test' sheet. Book an adult and a child.</t>
+        </is>
+      </c>
+      <c r="H126" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Open the seat map and select the CHILD.
+2. Click a seat marked 'Leg space seat'.
+3. Try to book it.
+4. Switch to the adult and click the same seat.</t>
+        </is>
+      </c>
+      <c r="I126" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The leg space seat is selectable for the child (Book &lt;seat&gt; for &lt;child&gt; is offered), as it is for the adult.</t>
+        </is>
+      </c>
+      <c r="J126" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K126" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Supplier rule stated by the business (Hussein, 28 Oct 2026): an adult holding an infant CAN select a leg space seat on the seat map (Admin and Portal), but Book / Hold / Pay after Hold with it is refused - Portal: In Progress, Admin: Failed - and the wallet is not charged. A CHILD may have a leg space seat: the booking is Confirmed and the wallet charged. Applies only to suppliers with the rule no-leg-space-seat-inf.</t>
+        </is>
+      </c>
+      <c r="L126" s="3" t="n"/>
+      <c r="M126" s="4" t="n"/>
+      <c r="N126" s="4" t="n"/>
+      <c r="O126" s="4" t="n"/>
+      <c r="P126" s="4" t="n"/>
+      <c r="Q126" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seat</t>
+        </is>
+      </c>
+      <c r="R126" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no-leg-space-seat-inf</t>
+        </is>
+      </c>
+      <c r="S126" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="T126" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">05 1 adult + 1 child - one-way, Economy</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="150" customHeight="1">
+      <c r="A127" s="2" t="n">
+        <v>126</v>
+      </c>
+      <c r="B127" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-SM-LEG-002</t>
+        </is>
+      </c>
+      <c r="C127" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y. Leg space seats</t>
+        </is>
+      </c>
+      <c r="D127" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">An adult holding an infant CAN select a leg space seat on the seat map</t>
+        </is>
+      </c>
+      <c r="E127" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The seat map does not stop it: the leg space rule is enforced when the booking is submitted (TC-SM-LEG-003, 005).</t>
+        </is>
+      </c>
+      <c r="F127" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="G127" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">See the 'Before every test' sheet. Book one adult with one infant.</t>
+        </is>
+      </c>
+      <c r="H127" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Open the seat map and select the adult who holds the infant.
+2. Click a seat marked 'Leg space seat'.
+3. Try to book it.</t>
+        </is>
+      </c>
+      <c r="I127" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">At least one leg space seat is selectable for the adult holding the infant.
+The refusal comes only at Book / Hold.</t>
+        </is>
+      </c>
+      <c r="J127" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K127" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Supplier rule stated by the business (Hussein, 28 Oct 2026): an adult holding an infant CAN select a leg space seat on the seat map (Admin and Portal), but Book / Hold / Pay after Hold with it is refused - Portal: In Progress, Admin: Failed - and the wallet is not charged. A CHILD may have a leg space seat: the booking is Confirmed and the wallet charged. Applies only to suppliers with the rule no-leg-space-seat-inf.</t>
+        </is>
+      </c>
+      <c r="L127" s="3" t="n"/>
+      <c r="M127" s="4" t="n"/>
+      <c r="N127" s="4" t="n"/>
+      <c r="O127" s="4" t="n"/>
+      <c r="P127" s="4" t="n"/>
+      <c r="Q127" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seat</t>
+        </is>
+      </c>
+      <c r="R127" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no-leg-space-seat-inf</t>
+        </is>
+      </c>
+      <c r="S127" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="T127" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">06 1 adult + 1 infant - one-way, Economy</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="150" customHeight="1">
+      <c r="A128" s="2" t="n">
+        <v>127</v>
+      </c>
+      <c r="B128" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-SM-LEG-003</t>
+        </is>
+      </c>
+      <c r="C128" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y. Leg space seats (SPENDS REAL MONEY if the rule is not enforced)</t>
+        </is>
+      </c>
+      <c r="D128" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Booking an infant-holding adult on a leg space seat is refused</t>
+        </is>
+      </c>
+      <c r="E128" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The rule is enforced when the booking is made: the airline does not complete it.</t>
+        </is>
+      </c>
+      <c r="F128" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="G128" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">See the 'Before every test' sheet. Book one adult with one infant.</t>
+        </is>
+      </c>
+      <c r="H128" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Open the seat map, select the adult holding the infant and book a seat marked 'Leg space seat' for them.
+2. Confirm the seats and press Book.
+3. Read the booking status and the wallet.</t>
+        </is>
+      </c>
+      <c r="I128" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Portal: the booking status is 'In Progress'. Admin: the booking status is 'Failed'.
+The wallet is NOT charged on either.</t>
+        </is>
+      </c>
+      <c r="J128" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partly</t>
+        </is>
+      </c>
+      <c r="K128" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Supplier rule stated by the business (Hussein, 28 Oct 2026): an adult holding an infant CAN select a leg space seat on the seat map (Admin and Portal), but Book / Hold / Pay after Hold with it is refused - Portal: In Progress, Admin: Failed - and the wallet is not charged. A CHILD may have a leg space seat: the booking is Confirmed and the wallet charged. Applies only to suppliers with the rule no-leg-space-seat-inf.</t>
+        </is>
+      </c>
+      <c r="L128" s="3" t="n"/>
+      <c r="M128" s="4" t="n"/>
+      <c r="N128" s="4" t="n"/>
+      <c r="O128" s="4" t="n"/>
+      <c r="P128" s="4" t="n"/>
+      <c r="Q128" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seat</t>
+        </is>
+      </c>
+      <c r="R128" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no-leg-space-seat-inf</t>
+        </is>
+      </c>
+      <c r="S128" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="T128" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20 Leg space rule at Book - 1 adult + 1 infant, adult on a leg space seat (SPENDS REAL MONEY if not enforced)</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="150" customHeight="1">
+      <c r="A129" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="B129" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-SM-LEG-004</t>
+        </is>
+      </c>
+      <c r="C129" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y. Leg space seats (SPENDS REAL MONEY if the rule is not enforced)</t>
+        </is>
+      </c>
+      <c r="D129" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Booking a child on a leg space seat is confirmed</t>
+        </is>
+      </c>
+      <c r="E129" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A child may have a leg space seat: the booking completes normally.</t>
+        </is>
+      </c>
+      <c r="F129" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="G129" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">See the 'Before every test' sheet. Book one adult and one child.</t>
+        </is>
+      </c>
+      <c r="H129" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Open the seat map, select the CHILD and book a seat marked 'Leg space seat' for them.
+2. Confirm the seats and press Book.
+3. Read the booking status and the wallet.</t>
+        </is>
+      </c>
+      <c r="I129" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The booking status is 'Confirmed'.
+The wallet is charged the quoted amount.</t>
+        </is>
+      </c>
+      <c r="J129" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partly</t>
+        </is>
+      </c>
+      <c r="K129" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Supplier rule stated by the business (Hussein, 28 Oct 2026): an adult holding an infant CAN select a leg space seat on the seat map (Admin and Portal), but Book / Hold / Pay after Hold with it is refused - Portal: In Progress, Admin: Failed - and the wallet is not charged. A CHILD may have a leg space seat: the booking is Confirmed and the wallet charged. Applies only to suppliers with the rule no-leg-space-seat-inf.</t>
+        </is>
+      </c>
+      <c r="L129" s="3" t="n"/>
+      <c r="M129" s="4" t="n"/>
+      <c r="N129" s="4" t="n"/>
+      <c r="O129" s="4" t="n"/>
+      <c r="P129" s="4" t="n"/>
+      <c r="Q129" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seat</t>
+        </is>
+      </c>
+      <c r="R129" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no-leg-space-seat-inf</t>
+        </is>
+      </c>
+      <c r="S129" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="T129" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">21 Leg space rule at Book - 1 adult + 1 child, child on a leg space seat (SPENDS REAL MONEY if not enforced)</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="150" customHeight="1">
+      <c r="A130" s="2" t="n">
+        <v>129</v>
+      </c>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-SM-LEG-005</t>
+        </is>
+      </c>
+      <c r="C130" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y. Leg space seats (SPENDS REAL MONEY if the rule is not enforced)</t>
+        </is>
+      </c>
+      <c r="D130" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Holding a booking with a leg space seat for an infant-holding adult is refused</t>
+        </is>
+      </c>
+      <c r="E130" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The rule is enforced at Hold as well as at Book: the airline does not hold it.</t>
+        </is>
+      </c>
+      <c r="F130" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="G130" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">See the 'Before every test' sheet. Book one adult with one infant.</t>
+        </is>
+      </c>
+      <c r="H130" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Open the seat map, select the adult holding the infant and book a seat marked 'Leg space seat' for them.
+2. Confirm the seats and press Hold.
+3. Read the booking status and the wallet.</t>
+        </is>
+      </c>
+      <c r="I130" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Portal: the booking status is 'In Progress' (not On Hold). Admin: the booking status is 'Failed'.
+The wallet is NOT charged on either.</t>
+        </is>
+      </c>
+      <c r="J130" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partly</t>
+        </is>
+      </c>
+      <c r="K130" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Supplier rule stated by the business (Hussein, 28 Oct 2026): an adult holding an infant CAN select a leg space seat on the seat map (Admin and Portal), but Book / Hold / Pay after Hold with it is refused - Portal: In Progress, Admin: Failed - and the wallet is not charged. A CHILD may have a leg space seat: the booking is Confirmed and the wallet charged. Applies only to suppliers with the rule no-leg-space-seat-inf.</t>
+        </is>
+      </c>
+      <c r="L130" s="3" t="n"/>
+      <c r="M130" s="4" t="n"/>
+      <c r="N130" s="4" t="n"/>
+      <c r="O130" s="4" t="n"/>
+      <c r="P130" s="4" t="n"/>
+      <c r="Q130" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hold + Seat</t>
+        </is>
+      </c>
+      <c r="R130" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no-leg-space-seat-inf</t>
+        </is>
+      </c>
+      <c r="S130" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="T130" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">22 Leg space rule at Hold - 1 adult + 1 infant, adult on a leg space seat</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T125"/>
+  <autoFilter ref="A1:T130"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>

</xml_diff>